<commit_message>
v1.7.1 add change language on setting
</commit_message>
<xml_diff>
--- a/src/locales/translations.xlsx
+++ b/src/locales/translations.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\condo-web\src\locales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FAC4A3-8BAD-4619-A7F4-9203856B1118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C67A9DF-6E81-4250-973F-B64A5112DE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcOnSave="0"/>
+  <calcPr calcId="191029" iterateDelta="1.0000000000000001E-5" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="244">
   <si>
     <t>id</t>
   </si>
@@ -588,6 +588,186 @@
   </si>
   <si>
     <t>写真を追加</t>
+  </si>
+  <si>
+    <t>stang</t>
+  </si>
+  <si>
+    <t>Stang</t>
+  </si>
+  <si>
+    <t>everyStangMatters</t>
+  </si>
+  <si>
+    <t>Every Stang Matters.</t>
+  </si>
+  <si>
+    <t>สตางค์</t>
+  </si>
+  <si>
+    <t>ทุกสตางค์มีความหมาย</t>
+  </si>
+  <si>
+    <t>selectPaidBy</t>
+  </si>
+  <si>
+    <t>Select Paid By</t>
+  </si>
+  <si>
+    <t>เลือกผู้ชำระเงิน</t>
+  </si>
+  <si>
+    <t>selectType</t>
+  </si>
+  <si>
+    <t>Select Type</t>
+  </si>
+  <si>
+    <t>เลือกประเภท</t>
+  </si>
+  <si>
+    <t>Installment Plan</t>
+  </si>
+  <si>
+    <t>แผนการผ่อนชำระ</t>
+  </si>
+  <si>
+    <t>installmentPlan</t>
+  </si>
+  <si>
+    <t>Generate</t>
+  </si>
+  <si>
+    <t>generate</t>
+  </si>
+  <si>
+    <t>สร้าง</t>
+  </si>
+  <si>
+    <t>Edit Type</t>
+  </si>
+  <si>
+    <t>แก้ไขประเภท</t>
+  </si>
+  <si>
+    <t>editType</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>แก้ไข</t>
+  </si>
+  <si>
+    <t>expression</t>
+  </si>
+  <si>
+    <t>result</t>
+  </si>
+  <si>
+    <t>Expression</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>คำอธิบาย</t>
+  </si>
+  <si>
+    <t>ผลลัพธ์</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Clear</t>
+  </si>
+  <si>
+    <t>ตกลง</t>
+  </si>
+  <si>
+    <t>ล้าง</t>
+  </si>
+  <si>
+    <t>noRecordFound</t>
+  </si>
+  <si>
+    <t>No Record Found</t>
+  </si>
+  <si>
+    <t>ไม่พบข้อมูล</t>
+  </si>
+  <si>
+    <t>changeLanguage</t>
+  </si>
+  <si>
+    <t>Change Language</t>
+  </si>
+  <si>
+    <t>เปลี่ยนภาษา</t>
+  </si>
+  <si>
+    <t>theme</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>Dark theme is active</t>
+  </si>
+  <si>
+    <t>Light theme is active</t>
+  </si>
+  <si>
+    <t>darkThemeIsActive</t>
+  </si>
+  <si>
+    <t>lightThemeIsActive</t>
+  </si>
+  <si>
+    <t>โหมด</t>
+  </si>
+  <si>
+    <t>โหมดมืดถูกใช้งาน</t>
+  </si>
+  <si>
+    <t>โหมดสว่างถูกใช้งาน</t>
+  </si>
+  <si>
+    <t>Switch to</t>
+  </si>
+  <si>
+    <t>switchTo</t>
+  </si>
+  <si>
+    <t>เปลี่ยนเป็น</t>
+  </si>
+  <si>
+    <t>Light Theme</t>
+  </si>
+  <si>
+    <t>Dark Theme</t>
+  </si>
+  <si>
+    <t>lightTheme</t>
+  </si>
+  <si>
+    <t>darkTheme</t>
+  </si>
+  <si>
+    <t>โหมดสว่าง</t>
+  </si>
+  <si>
+    <t>โหมดมืด</t>
   </si>
 </sst>
 </file>
@@ -959,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EFFCAA-6DA9-40A3-BF28-CA3BC524DD9C}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1591,6 +1771,226 @@
         <v>183</v>
       </c>
     </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>184</v>
+      </c>
+      <c r="B38" t="s">
+        <v>185</v>
+      </c>
+      <c r="C38" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>186</v>
+      </c>
+      <c r="B39" t="s">
+        <v>187</v>
+      </c>
+      <c r="C39" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>190</v>
+      </c>
+      <c r="B40" t="s">
+        <v>191</v>
+      </c>
+      <c r="C40" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>193</v>
+      </c>
+      <c r="B41" t="s">
+        <v>194</v>
+      </c>
+      <c r="C41" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>198</v>
+      </c>
+      <c r="B42" t="s">
+        <v>196</v>
+      </c>
+      <c r="C42" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>200</v>
+      </c>
+      <c r="B43" t="s">
+        <v>199</v>
+      </c>
+      <c r="C43" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>204</v>
+      </c>
+      <c r="B44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C44" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>205</v>
+      </c>
+      <c r="B45" t="s">
+        <v>206</v>
+      </c>
+      <c r="C45" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>208</v>
+      </c>
+      <c r="B46" t="s">
+        <v>210</v>
+      </c>
+      <c r="C46" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>209</v>
+      </c>
+      <c r="B47" t="s">
+        <v>211</v>
+      </c>
+      <c r="C47" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>214</v>
+      </c>
+      <c r="B48" t="s">
+        <v>216</v>
+      </c>
+      <c r="C48" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>215</v>
+      </c>
+      <c r="B49" t="s">
+        <v>217</v>
+      </c>
+      <c r="C49" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>220</v>
+      </c>
+      <c r="B50" t="s">
+        <v>221</v>
+      </c>
+      <c r="C50" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>223</v>
+      </c>
+      <c r="B51" t="s">
+        <v>224</v>
+      </c>
+      <c r="C51" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>226</v>
+      </c>
+      <c r="B52" t="s">
+        <v>227</v>
+      </c>
+      <c r="C52" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>230</v>
+      </c>
+      <c r="B53" t="s">
+        <v>228</v>
+      </c>
+      <c r="C53" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>231</v>
+      </c>
+      <c r="B54" t="s">
+        <v>229</v>
+      </c>
+      <c r="C54" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>236</v>
+      </c>
+      <c r="B55" t="s">
+        <v>235</v>
+      </c>
+      <c r="C55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>240</v>
+      </c>
+      <c r="B56" t="s">
+        <v>238</v>
+      </c>
+      <c r="C56" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>241</v>
+      </c>
+      <c r="B57" t="s">
+        <v>239</v>
+      </c>
+      <c r="C57" t="s">
+        <v>243</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
v1.8.0 add calendar memo and tag
</commit_message>
<xml_diff>
--- a/src/locales/translations.xlsx
+++ b/src/locales/translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\condo-web\src\locales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8E4AEC-9350-48BB-83AA-0B593218DEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EAAF4AD-AB4B-4EC4-A739-A93DEF4F8DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="355">
   <si>
     <t>id</t>
   </si>
@@ -939,16 +939,184 @@
   </si>
   <si>
     <t>ทดสอบ</t>
+  </si>
+  <si>
+    <t>today</t>
+  </si>
+  <si>
+    <t>Today</t>
+  </si>
+  <si>
+    <t>วันนี้</t>
+  </si>
+  <si>
+    <t>sun</t>
+  </si>
+  <si>
+    <t>mon</t>
+  </si>
+  <si>
+    <t>tue</t>
+  </si>
+  <si>
+    <t>wed</t>
+  </si>
+  <si>
+    <t>thu</t>
+  </si>
+  <si>
+    <t>sat</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>Thu</t>
+  </si>
+  <si>
+    <t>Sat</t>
+  </si>
+  <si>
+    <t>อา</t>
+  </si>
+  <si>
+    <t>จ</t>
+  </si>
+  <si>
+    <t>อ</t>
+  </si>
+  <si>
+    <t>พ</t>
+  </si>
+  <si>
+    <t>พฤ</t>
+  </si>
+  <si>
+    <t>ศ</t>
+  </si>
+  <si>
+    <t>ส</t>
+  </si>
+  <si>
+    <t>fri</t>
+  </si>
+  <si>
+    <t>Fri</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>December</t>
+  </si>
+  <si>
+    <t>มกราคม</t>
+  </si>
+  <si>
+    <t>กุมภาพันธ์</t>
+  </si>
+  <si>
+    <t>มีนาคม</t>
+  </si>
+  <si>
+    <t>เมษายน</t>
+  </si>
+  <si>
+    <t>พฤษภาคม</t>
+  </si>
+  <si>
+    <t>มิถุนายน</t>
+  </si>
+  <si>
+    <t>กรกฏาคม</t>
+  </si>
+  <si>
+    <t>สิงหาคม</t>
+  </si>
+  <si>
+    <t>กันยายน</t>
+  </si>
+  <si>
+    <t>ตุลาคม</t>
+  </si>
+  <si>
+    <t>พฤศจิกายน</t>
+  </si>
+  <si>
+    <t>ธันวาคม</t>
+  </si>
+  <si>
+    <t>tag</t>
+  </si>
+  <si>
+    <t>Tag</t>
+  </si>
+  <si>
+    <t>แท็ก</t>
+  </si>
+  <si>
+    <t>payerOtherAmount</t>
+  </si>
+  <si>
+    <t>Payer/Other Amount</t>
+  </si>
+  <si>
+    <t>ของผู้จ่าย/ของคนอื่น</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1311,7 +1479,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EFFCAA-6DA9-40A3-BF28-CA3BC524DD9C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -2388,7 +2556,250 @@
         <v>300</v>
       </c>
     </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>301</v>
+      </c>
+      <c r="B78" t="s">
+        <v>302</v>
+      </c>
+      <c r="C78" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>304</v>
+      </c>
+      <c r="B79" t="s">
+        <v>310</v>
+      </c>
+      <c r="C79" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>305</v>
+      </c>
+      <c r="B80" t="s">
+        <v>311</v>
+      </c>
+      <c r="C80" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>306</v>
+      </c>
+      <c r="B81" t="s">
+        <v>312</v>
+      </c>
+      <c r="C81" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>307</v>
+      </c>
+      <c r="B82" t="s">
+        <v>313</v>
+      </c>
+      <c r="C82" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>308</v>
+      </c>
+      <c r="B83" t="s">
+        <v>314</v>
+      </c>
+      <c r="C83" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>323</v>
+      </c>
+      <c r="B84" t="s">
+        <v>324</v>
+      </c>
+      <c r="C84" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>309</v>
+      </c>
+      <c r="B85" t="s">
+        <v>315</v>
+      </c>
+      <c r="C85" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>325</v>
+      </c>
+      <c r="B86" t="s">
+        <v>325</v>
+      </c>
+      <c r="C86" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>327</v>
+      </c>
+      <c r="B87" t="s">
+        <v>327</v>
+      </c>
+      <c r="C87" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>326</v>
+      </c>
+      <c r="B88" t="s">
+        <v>326</v>
+      </c>
+      <c r="C88" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>328</v>
+      </c>
+      <c r="B89" t="s">
+        <v>328</v>
+      </c>
+      <c r="C89" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>329</v>
+      </c>
+      <c r="B90" t="s">
+        <v>329</v>
+      </c>
+      <c r="C90" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>330</v>
+      </c>
+      <c r="B91" t="s">
+        <v>330</v>
+      </c>
+      <c r="C91" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>331</v>
+      </c>
+      <c r="B92" t="s">
+        <v>331</v>
+      </c>
+      <c r="C92" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>332</v>
+      </c>
+      <c r="B93" t="s">
+        <v>332</v>
+      </c>
+      <c r="C93" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>333</v>
+      </c>
+      <c r="B94" t="s">
+        <v>333</v>
+      </c>
+      <c r="C94" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>334</v>
+      </c>
+      <c r="B95" t="s">
+        <v>334</v>
+      </c>
+      <c r="C95" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>335</v>
+      </c>
+      <c r="B96" t="s">
+        <v>335</v>
+      </c>
+      <c r="C96" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>336</v>
+      </c>
+      <c r="B97" t="s">
+        <v>336</v>
+      </c>
+      <c r="C97" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>349</v>
+      </c>
+      <c r="B98" t="s">
+        <v>350</v>
+      </c>
+      <c r="C98" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>352</v>
+      </c>
+      <c r="B99" t="s">
+        <v>353</v>
+      </c>
+      <c r="C99" t="s">
+        <v>354</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.1 add manage tag on calendar
</commit_message>
<xml_diff>
--- a/src/locales/translations.xlsx
+++ b/src/locales/translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\condo-web\src\locales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EAAF4AD-AB4B-4EC4-A739-A93DEF4F8DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCF1296-5E19-4819-AF4B-5199F437A9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="361">
   <si>
     <t>id</t>
   </si>
@@ -1101,6 +1101,24 @@
   </si>
   <si>
     <t>ของผู้จ่าย/ของคนอื่น</t>
+  </si>
+  <si>
+    <t>editTag</t>
+  </si>
+  <si>
+    <t>Edit Tag</t>
+  </si>
+  <si>
+    <t>แก้ไขแท็ก</t>
+  </si>
+  <si>
+    <t>noTag</t>
+  </si>
+  <si>
+    <t>No Tag</t>
+  </si>
+  <si>
+    <t>ไม่มีแท็ก</t>
   </si>
 </sst>
 </file>
@@ -1479,7 +1497,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EFFCAA-6DA9-40A3-BF28-CA3BC524DD9C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -2798,6 +2816,28 @@
         <v>354</v>
       </c>
     </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>355</v>
+      </c>
+      <c r="B100" t="s">
+        <v>356</v>
+      </c>
+      <c r="C100" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>358</v>
+      </c>
+      <c r="B101" t="s">
+        <v>359</v>
+      </c>
+      <c r="C101" t="s">
+        <v>360</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
v1.9.0 add register and buddy
</commit_message>
<xml_diff>
--- a/src/locales/translations.xlsx
+++ b/src/locales/translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\condo-web\src\locales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8666D4C-FF69-4CC4-BABA-98480369C771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD88DC6-2002-41F0-B43B-542FE88031A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="381">
   <si>
     <t>id</t>
   </si>
@@ -1154,13 +1154,31 @@
     <t>You have buddy now.</t>
   </si>
   <si>
-    <t>คูณมีคู่หูแล้ว</t>
-  </si>
-  <si>
     <t>by</t>
   </si>
   <si>
     <t>โดย</t>
+  </si>
+  <si>
+    <t>register</t>
+  </si>
+  <si>
+    <t>Register</t>
+  </si>
+  <si>
+    <t>สมัคร</t>
+  </si>
+  <si>
+    <t>confirmPassword</t>
+  </si>
+  <si>
+    <t>Confirm Password</t>
+  </si>
+  <si>
+    <t>ยืนยันรหัสผ่าน</t>
+  </si>
+  <si>
+    <t>คุณมีคู่หูแล้ว</t>
   </si>
 </sst>
 </file>
@@ -1539,7 +1557,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EFFCAA-6DA9-40A3-BF28-CA3BC524DD9C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -2921,18 +2939,40 @@
         <v>371</v>
       </c>
       <c r="C105" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
+        <v>372</v>
+      </c>
+      <c r="B106" t="s">
+        <v>372</v>
+      </c>
+      <c r="C106" t="s">
         <v>373</v>
       </c>
-      <c r="B106" t="s">
-        <v>373</v>
-      </c>
-      <c r="C106" t="s">
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
         <v>374</v>
+      </c>
+      <c r="B107" t="s">
+        <v>375</v>
+      </c>
+      <c r="C107" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>377</v>
+      </c>
+      <c r="B108" t="s">
+        <v>378</v>
+      </c>
+      <c r="C108" t="s">
+        <v>379</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v1.9.10 add animation for all
</commit_message>
<xml_diff>
--- a/src/locales/translations.xlsx
+++ b/src/locales/translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\condo\condo-web\src\locales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB84D6B8-CF52-43DD-8A4F-C227E220FEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6854802F-5571-4825-A0EF-BF98C96A558A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{B932D239-48A5-4026-8CCD-CA2BFDECA8AC}"/>
   </bookViews>
   <sheets>
     <sheet name="DATA" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="402">
   <si>
     <t>id</t>
   </si>
@@ -1215,6 +1215,33 @@
   </si>
   <si>
     <t>userInstallmentPlan</t>
+  </si>
+  <si>
+    <t>currentPassword</t>
+  </si>
+  <si>
+    <t>newPassword</t>
+  </si>
+  <si>
+    <t>รหัสผ่านปัจจุบัน</t>
+  </si>
+  <si>
+    <t>รหัสผ่านใหม่</t>
+  </si>
+  <si>
+    <t>Current Password</t>
+  </si>
+  <si>
+    <t>New Password</t>
+  </si>
+  <si>
+    <t>confirm</t>
+  </si>
+  <si>
+    <t>Confirm</t>
+  </si>
+  <si>
+    <t>ยืนยัน</t>
   </si>
 </sst>
 </file>
@@ -1593,7 +1620,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01EFFCAA-6DA9-40A3-BF28-CA3BC524DD9C}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -3055,6 +3082,39 @@
         <v>391</v>
       </c>
     </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>393</v>
+      </c>
+      <c r="B113" t="s">
+        <v>397</v>
+      </c>
+      <c r="C113" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>394</v>
+      </c>
+      <c r="B114" t="s">
+        <v>398</v>
+      </c>
+      <c r="C114" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>399</v>
+      </c>
+      <c r="B115" t="s">
+        <v>400</v>
+      </c>
+      <c r="C115" t="s">
+        <v>401</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>